<commit_message>
test(xlsx): use the reporter's own workbook as the #395 fixture
The file attached to the issue has a shape the stand-in did not: its empty
merge is `B1:N1`, above the only value (`A2`) and to the *right* of it, so the
row axis underflows while the column axis has to grow out to column N. The
stand-in merged from column A and only exercised growing upward.

Swapped into the corpus in place of the stand-in, and the geometry is pinned by
its own unit test next to the existing one. The file converts to the single
1x1 table its one value makes; the empty merge contributes nothing, as it does
in docling.

Refs #395

Signed-off-by: artiz <artem.kustikov@gmail.com>
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EY5KAiquN4YpVf2PXEQkVT
</commit_message>
<xml_diff>
--- a/crates/docling/tests/data/xlsx/sources/xlsx_empty_merge_before_data.xlsx
+++ b/crates/docling/tests/data/xlsx/sources/xlsx_empty_merge_before_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,35 +413,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>data</t>
         </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Bolt</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>